<commit_message>
Normalize network planning form template; remove GSK-specific data
Replace GSK customer names, real subscription ID, and corp IP ranges with generic placeholders so the template is reusable for any customer.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: 85b5fd6b-41f5-4dc3-baf1-ba40df9c8691
</commit_message>
<xml_diff>
--- a/utilities/onboarding-tool/scripts/stage1-planning/network-planning-form-template.xlsx
+++ b/utilities/onboarding-tool/scripts/stage1-planning/network-planning-form-template.xlsx
@@ -645,10 +645,11 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Fill the Value column (yellow). Column A tags are stable — do not rename. SUBNET/POLICY/WAIVER rows may be added or removed. Yellow example values are GSK-derived; overwrite them.</t>
-        </is>
-      </c>
-    </row>
+          <t>Fill the Value column (yellow). Column A tags are stable — do not rename. SUBNET/POLICY/WAIVER rows may be added or removed. Yellow example values are illustrative; overwrite them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -704,7 +705,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>67e7fe44-d943-4033-8f1f-742a9b0e6859</t>
+          <t>00000000-0000-0000-0000-000000000000</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -847,7 +848,7 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>rd-research-network-vnet-devtest</t>
+          <t>network-rg</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
@@ -943,12 +944,10 @@
           <t>network.existingSubnets</t>
         </is>
       </c>
-      <c r="B22" s="19" t="inlineStr"/>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>Comma-separated CIDRs already in use in the VNet (overlap check). FR1.3</t>
-        </is>
-      </c>
+      <c r="B22" s="22" t="n"/>
+      <c r="C22" s="22" t="n"/>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="23" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
@@ -1125,26 +1124,10 @@
           <t>SUBNET</t>
         </is>
       </c>
-      <c r="B30" s="19" t="inlineStr">
-        <is>
-          <t>spare</t>
-        </is>
-      </c>
-      <c r="C30" s="19" t="inlineStr">
-        <is>
-          <t>10.46.253.64/27</t>
-        </is>
-      </c>
-      <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>/27</t>
-        </is>
-      </c>
-      <c r="E30" s="19" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+      <c r="B30" s="22" t="n"/>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="23" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
@@ -1189,16 +1172,10 @@
           <t>storage.access</t>
         </is>
       </c>
-      <c r="B34" s="19" t="inlineStr">
-        <is>
-          <t>privateEndpoint</t>
-        </is>
-      </c>
-      <c r="E34" s="20" t="inlineStr">
-        <is>
-          <t>privateEndpoint | serviceEndpoint</t>
-        </is>
-      </c>
+      <c r="B34" s="22" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="23" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
@@ -1281,16 +1258,10 @@
           <t>deployMode</t>
         </is>
       </c>
-      <c r="B40" s="19" t="inlineStr">
-        <is>
-          <t>GlobalStandard</t>
-        </is>
-      </c>
-      <c r="E40" s="20" t="inlineStr">
-        <is>
-          <t>GlobalStandard | DataZoneStandard (data residency). FR1.5</t>
-        </is>
-      </c>
+      <c r="B40" s="22" t="n"/>
+      <c r="C40" s="22" t="n"/>
+      <c r="D40" s="22" t="n"/>
+      <c r="E40" s="23" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
@@ -1307,7 +1278,7 @@
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>gsk-rd-disc-ws</t>
+          <t>disc-ws</t>
         </is>
       </c>
       <c r="E42" s="20" t="inlineStr">
@@ -1324,7 +1295,7 @@
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>gsk-rd-p1</t>
+          <t>project1</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -1341,7 +1312,7 @@
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>gsk-rd-sc</t>
+          <t>disc-sc</t>
         </is>
       </c>
       <c r="E44" s="20" t="inlineStr">
@@ -1441,16 +1412,10 @@
           <t>names.investigation</t>
         </is>
       </c>
-      <c r="B50" s="19" t="inlineStr">
-        <is>
-          <t>hero-inv</t>
-        </is>
-      </c>
-      <c r="E50" s="20" t="inlineStr">
-        <is>
-          <t>1-20.</t>
-        </is>
-      </c>
+      <c r="B50" s="22" t="n"/>
+      <c r="C50" s="22" t="n"/>
+      <c r="D50" s="22" t="n"/>
+      <c r="E50" s="23" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
@@ -1477,11 +1442,10 @@
           <t>POLICY</t>
         </is>
       </c>
-      <c r="B53" s="19" t="inlineStr">
-        <is>
-          <t>Storage accounts should disable public network access</t>
-        </is>
-      </c>
+      <c r="B53" s="22" t="n"/>
+      <c r="C53" s="22" t="n"/>
+      <c r="D53" s="22" t="n"/>
+      <c r="E53" s="23" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="17" t="inlineStr">
@@ -1567,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C20"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1575,20 +1539,22 @@
     <col width="95" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Network Planning Form — GSK RD Research (devtest)</t>
+          <t>Network Planning Form — Customer / Workload (devtest)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Populated from the customer BYO-VNet snapshot: gsk-rd-research-devtest-us6-vnet002 (East US 2).</t>
-        </is>
-      </c>
-    </row>
+          <t>Populated from the customer BYO-VNet snapshot: customer-vnet (East US 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -1597,7 +1563,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>GSK RD Research — Discovery/Foundry on customer-provided VNet</t>
+          <t>Customer / Workload — Discovery/Foundry on customer-provided VNet</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1611,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>gsk-rd-research-applications-devtest</t>
+          <t>customer-subscription</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1623,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>67e7fe44-d943-4033-8f1f-742a9b0e6859</t>
+          <t>00000000-0000-0000-0000-000000000000</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1659,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>rd-research-network-vnet-devtest</t>
+          <t>network-rg</t>
         </is>
       </c>
     </row>
@@ -1709,6 +1675,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
@@ -1724,7 +1691,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Azure portal screenshots in discovery-doc/bicep/GSK-Network (vnet subnets, 3 container-app NSGs, route table rt001).</t>
+          <t>Network export / portal screenshots of the customer VNet, subnets, NSGs, and route tables.</t>
         </is>
       </c>
     </row>
@@ -1785,14 +1752,14 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Network Topology Diagram — GSK RD Research (devtest, East US 2)</t>
+          <t>Network Topology Diagram — Customer / Workload (devtest, East US 2)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from the GSK-Network portal snapshot. See sheets 1-5 for tabular detail.</t>
+          <t>Generated from the customer network portal snapshot. See sheets 1-5 for tabular detail.</t>
         </is>
       </c>
     </row>
@@ -1837,6 +1804,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1879,7 +1847,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>0.0.0.0/0 -&gt; NVA 10.42.157.126 (egress firewall). RFC1918 (10/8, 11/8, 172.16/12, 192.168/16), internal subnet CIDRs, GSK corp public ranges, and Google restricted-API CIDRs (199.36.153.4/30, .8/30) -&gt; NVA 10.42.156.126.</t>
+          <t>0.0.0.0/0 -&gt; NVA 10.42.157.126 (egress firewall). RFC1918 (10/8, 11/8, 172.16/12, 192.168/16), internal subnet CIDRs, Corp public ranges, and Google restricted-API CIDRs (199.36.153.4/30, .8/30) -&gt; NVA 10.42.156.126.</t>
         </is>
       </c>
       <c r="C6" s="22" t="n"/>
@@ -1913,7 +1881,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Inbound allowed from GSK corp ranges (192.154.93.0/24, 192.154.91.0/24, ...) per NSG rule 'inbound-gsk'.</t>
+          <t>Inbound allowed from corp ranges (&lt;corp-range-1&gt;, &lt;corp-range-2&gt;, ...) per NSG rule 'inbound-corp'.</t>
         </is>
       </c>
       <c r="C8" s="22" t="n"/>
@@ -1939,6 +1907,7 @@
       <c r="F9" s="22" t="n"/>
       <c r="G9" s="23" t="n"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
@@ -1986,7 +1955,7 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>gsk-rd-research-devtest-us6-vnet002</t>
+          <t>customer-vnet</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -1996,7 +1965,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>rd-research-network-vnet-devtest</t>
+          <t>network-rg</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -2387,6 +2356,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -2647,7 +2617,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>GSK corp 192.154.93.0/24, 192.154.91.0/24</t>
+          <t>Corp &lt;corp-range-1&gt;, &lt;corp-range-2&gt;</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -2667,7 +2637,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Inbound via NVA; NSG 'inbound-gsk' Allow</t>
+          <t>Inbound via NVA; NSG 'inbound-corp' Allow</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -2694,7 +2664,7 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>10/8,11/8,172.16/12,192.168/16, GSK public CIDRs, 199.36.153.4/30 &amp; .8/30</t>
+          <t>10/8,11/8,172.16/12,192.168/16, corp public CIDRs, 199.36.153.4/30 &amp; .8/30</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -2868,10 +2838,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>gsk-rd-research-devtest-us6-vnet002 — 8 subnets, each with an NSG and route table rt001 (forced tunneling).</t>
-        </is>
-      </c>
-    </row>
+          <t>customer-vnet — 8 subnets, each with an NSG and route table rt001 (forced tunneling).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -2914,7 +2885,7 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>gsk-rd-research-devtest-us6-vnet002</t>
+          <t>customer-vnet</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -2939,10 +2910,11 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>RG: rd-research-network-vnet-devtest</t>
-        </is>
-      </c>
-    </row>
+          <t>RG: network-rg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
@@ -3415,6 +3387,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -3543,12 +3516,12 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>inbound-gsk</t>
+          <t>inbound-corp</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>192.154.93.0/24,192.154.91.0/24,...</t>
+          <t>&lt;corp-range-1&gt;,&lt;corp-range-2&gt;,...</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
@@ -3578,7 +3551,7 @@
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>GSK corp mgmt inbound</t>
+          <t>Corp mgmt inbound</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3791,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>outbound-gsk</t>
+          <t>outbound-corp</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -3833,7 +3806,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>192.154.93.0/24,192.154.91.0/24,...</t>
+          <t>&lt;corp-range-1&gt;,&lt;corp-range-2&gt;,...</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
@@ -3853,7 +3826,7 @@
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>To GSK corp ranges</t>
+          <t>To corp ranges</t>
         </is>
       </c>
     </row>
@@ -4093,12 +4066,12 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>inbound-gsk</t>
+          <t>inbound-corp</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>192.154.93.0/24,192.154.91.0/24,...</t>
+          <t>&lt;corp-range-1&gt;,&lt;corp-range-2&gt;,...</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -4128,7 +4101,7 @@
       </c>
       <c r="K16" s="10" t="inlineStr">
         <is>
-          <t>GSK corp mgmt inbound</t>
+          <t>Corp mgmt inbound</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4341,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>outbound-gsk</t>
+          <t>outbound-corp</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -4383,7 +4356,7 @@
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>192.154.93.0/24,192.154.91.0/24,...</t>
+          <t>&lt;corp-range-1&gt;,&lt;corp-range-2&gt;,...</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
@@ -4403,7 +4376,7 @@
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
-          <t>To GSK corp ranges</t>
+          <t>To corp ranges</t>
         </is>
       </c>
     </row>
@@ -4643,12 +4616,12 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>inbound-gsk</t>
+          <t>inbound-corp</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>192.154.93.0/24,192.154.91.0/24,...</t>
+          <t>&lt;corp-range-1&gt;,&lt;corp-range-2&gt;,...</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -4678,7 +4651,7 @@
       </c>
       <c r="K26" s="10" t="inlineStr">
         <is>
-          <t>GSK corp mgmt inbound</t>
+          <t>Corp mgmt inbound</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4891,7 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>outbound-gsk</t>
+          <t>outbound-corp</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -4933,7 +4906,7 @@
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>192.154.93.0/24,192.154.91.0/24,...</t>
+          <t>&lt;corp-range-1&gt;,&lt;corp-range-2&gt;,...</t>
         </is>
       </c>
       <c r="H31" s="10" t="inlineStr">
@@ -4953,7 +4926,7 @@
       </c>
       <c r="K31" s="10" t="inlineStr">
         <is>
-          <t>To GSK corp ranges</t>
+          <t>To corp ranges</t>
         </is>
       </c>
     </row>
@@ -5249,6 +5222,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -5642,7 +5616,7 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>130.23.0.0/16, 139.136.0.0/16, 143.193.0.0/16, 145.240.0.0/16, 147.184.0.0/16, 152.51.0.0/16, 159.30.0.0/16, 159.114.0.0/16, 161.147.0.0/16, 166.71.0.0/16, 192.6.210.0/24, 192.30.61.0/24, 192.46.157.0/24, 192.55.202.0/24, 192.56.74.0/23, 192.81.190.0/24, 192.154.91-93.0/24, 193.53.6.0/24, 193.143.229.0/24, 194.13.2.0/23, 198.28.64.0/18, 199.28.0.0/16, 192.221.197.0/24, 192.246.19-20.0/24, 193.74.128.0/21, 193.130.44.0/24</t>
+          <t>&lt;corp public IP ranges&gt;</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -5657,7 +5631,7 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>GSK corp public ranges (intranet05..33)</t>
+          <t>Corp public ranges (intranet05..33)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Genericize planning form IPs; use clean 10.0.0.0/23 address plan
Remap all subnet CIDRs to a generic, non-overlapping 10.0.0.0/23 scheme and replace NVA next-hop IPs with generic hub addresses. Subnet CIDRs stay consistent across Config, topology, VNet/subnet, NSG, and route-table sheets.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: 85b5fd6b-41f5-4dc3-baf1-ba40df9c8691
</commit_message>
<xml_diff>
--- a/utilities/onboarding-tool/scripts/stage1-planning/network-planning-form-template.xlsx
+++ b/utilities/onboarding-tool/scripts/stage1-planning/network-planning-form-template.xlsx
@@ -865,7 +865,7 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>10.46.252.0/23</t>
+          <t>10.0.0.0/23</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>10.46.252.0/23</t>
+          <t>10.0.0.0/23</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>10.42.157.126</t>
+          <t>10.1.0.4</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>10.46.253.128/26</t>
+          <t>10.0.0.128/26</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>10.46.252.128/26</t>
+          <t>10.0.0.192/26</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>10.46.253.0/27</t>
+          <t>10.0.1.96/27</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>0.0.0.0/0 is routed to NVA 10.42.157.126, so the NSG 'AllowInternetOutBound' does NOT give direct egress — all Internet is inspected by the on-prem firewall. The NVA must allow AKS bootstrap (*.azureedge.net) + AzureCloud:443, or provisioning stalls.</t>
+          <t>0.0.0.0/0 is routed to NVA 10.1.0.4, so the NSG 'AllowInternetOutBound' does NOT give direct egress — all Internet is inspected by the on-prem firewall. The NVA must allow AKS bootstrap (*.azureedge.net) + AzureCloud:443, or provisioning stalls.</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>0.0.0.0/0 -&gt; NVA 10.42.157.126 (egress firewall). RFC1918 (10/8, 11/8, 172.16/12, 192.168/16), internal subnet CIDRs, Corp public ranges, and Google restricted-API CIDRs (199.36.153.4/30, .8/30) -&gt; NVA 10.42.156.126.</t>
+          <t>0.0.0.0/0 -&gt; NVA 10.1.0.4 (egress firewall). RFC1918 (10/8, 11/8, 172.16/12, 192.168/16), internal subnet CIDRs, Corp public ranges, and Google restricted-API CIDRs (199.36.153.4/30, .8/30) -&gt; NVA 10.1.0.5.</t>
         </is>
       </c>
       <c r="C6" s="22" t="n"/>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>None shown. Corp/on-prem reachability via the NVA next hops (10.42.156.126 / 10.42.157.126) which sit outside this VNet.</t>
+          <t>None shown. Corp/on-prem reachability via the NVA next hops (10.1.0.5 / 10.1.0.4) which sit outside this VNet.</t>
         </is>
       </c>
       <c r="C7" s="22" t="n"/>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>VNet 10.46.252.0/23 (inferred)</t>
+          <t>VNet 10.0.0.0/23 (inferred)</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.128/26</t>
+          <t>10.0.0.128/26</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26, .64/26, 10.46.253.32/27</t>
+          <t>10.0.0.0/26, 10.0.0.64/26, 10.0.1.64/27</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.0/27, 10.46.253.64/27</t>
+          <t>10.0.1.96/27, 10.0.1.128/27</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.128/26, .192/26</t>
+          <t>10.0.0.192/26, 10.0.1.0/26</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>next hop 10.42.157.126</t>
+          <t>next hop 10.1.0.4</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>next hop 10.42.156.126</t>
+          <t>next hop 10.1.0.5</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>UDR -&gt; NVA 10.42.157.126 (NOT direct)</t>
+          <t>UDR -&gt; NVA 10.1.0.4 (NOT direct)</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>UDR -&gt; NVA 10.42.157.126</t>
+          <t>UDR -&gt; NVA 10.1.0.4</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>UDR default -&gt; NVA 10.42.157.126</t>
+          <t>UDR default -&gt; NVA 10.1.0.4</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>UDR internal* -&gt; NVA 10.42.156.126</t>
+          <t>UDR internal* -&gt; NVA 10.1.0.5</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>UDR intranet*/gapi* -&gt; NVA 10.42.156.126</t>
+          <t>UDR intranet*/gapi* -&gt; NVA 10.1.0.5</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/23 (inferred — confirm)</t>
+          <t>10.0.0.0/23 (inferred — confirm)</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.128/26</t>
+          <t>10.0.0.128/26</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.128/26</t>
+          <t>10.0.0.192/26</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.192/26</t>
+          <t>10.0.1.0/26</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.0/27</t>
+          <t>10.0.1.96/27</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.64/27</t>
+          <t>10.0.1.128/27</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="H25" s="10" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="H26" s="10" t="inlineStr">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="H30" s="10" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
@@ -5218,7 +5218,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Route table rt001 — forced tunneling. Attached to all subnets. Default egress -&gt; NVA 10.42.157.126; everything else -&gt; 10.42.156.126.</t>
+          <t>Route table rt001 — forced tunneling. Attached to all subnets. Default egress -&gt; NVA 10.1.0.4; everything else -&gt; 10.1.0.5.</t>
         </is>
       </c>
     </row>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>10.42.157.126</t>
+          <t>10.1.0.4</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.0/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -5356,7 +5356,7 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -5373,7 +5373,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.64/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -5400,7 +5400,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.0/27</t>
+          <t>10.0.1.96/27</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -5427,7 +5427,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.32/27</t>
+          <t>10.0.1.64/27</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -5454,7 +5454,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>10.46.253.64/27</t>
+          <t>10.0.1.128/27</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>10.46.252.128/26</t>
+          <t>10.0.0.192/26</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>10.42.156.126</t>
+          <t>10.1.0.5</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">

</xml_diff>